<commit_message>
feat: Implement decimal separator configuration for Excel output to support regional formatting
</commit_message>
<xml_diff>
--- a/output/BBVA_VISA_20250613.xlsx
+++ b/output/BBVA_VISA_20250613.xlsx
@@ -471,12 +471,14 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D2" t="n">
-        <v>4940</v>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>4940,0</t>
+        </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>
@@ -496,12 +498,14 @@
           <t>ARS</t>
         </is>
       </c>
-      <c r="D3" t="n">
-        <v>15249.34</v>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>15249,34</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>BBVA VISA</t>
+          <t>BBVA Visa</t>
         </is>
       </c>
     </row>

</xml_diff>